<commit_message>
Feat/more studi ausbild richtungen (#558)
* Add more Studi&Ausbildungsrichtungen

* Update Docs

* Lint

* Update doc/docs/documentation/architecture/colorpalette/index.md

Co-authored-by: coderabbitai[bot] <136622811+coderabbitai[bot]@users.noreply.github.com>

* Update praktikumsplaner-frontend/src/components/praktikumsplaetze/Meldung/AusbildungsJahrSelect.vue

Co-authored-by: coderabbitai[bot] <136622811+coderabbitai[bot]@users.noreply.github.com>

* Fix FISI Color

* Zuweisungszeiten update

* Update doc/docs/documentation/architecture/colorpalette/index.md

Co-authored-by: coderabbitai[bot] <136622811+coderabbitai[bot]@users.noreply.github.com>

* Fix Select

* Update praktikumsplaner-frontend/src/types/Ausbildungsjahr.ts

Co-authored-by: coderabbitai[bot] <136622811+coderabbitai[bot]@users.noreply.github.com>

---------

Co-authored-by: coderabbitai[bot] <136622811+coderabbitai[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/doc/docs/public/assets/Import_Standart.xlsx
+++ b/doc/docs/public/assets/Import_Standart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luis.einig\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rene.zarwel\develop\Projekte\Praktikumsplaner\doc\docs\public\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07D1B78D-9D86-4328-BF89-219BA38F513A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCA5539F-50C7-4B0A-8E0D-2FAF2AD7A468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33180" yWindow="-525" windowWidth="28800" windowHeight="15375" xr2:uid="{E95CBEE5-BDCF-48D0-B574-A8FA4EA1B085}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E95CBEE5-BDCF-48D0-B574-A8FA4EA1B085}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -99,7 +99,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -117,12 +117,6 @@
       <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Segoe UI"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -210,9 +204,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -250,7 +244,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -356,7 +350,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -498,7 +492,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -518,16 +512,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C40CCF9E-2FB7-4310-91B7-7540413BFD8B}">
   <dimension ref="A1:E20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.796875" customWidth="1"/>
-    <col min="2" max="2" width="16.69921875" customWidth="1"/>
-    <col min="3" max="3" width="15.796875" customWidth="1"/>
-    <col min="4" max="4" width="18.09765625" customWidth="1"/>
-    <col min="5" max="5" width="20.8984375" customWidth="1"/>
+    <col min="1" max="1" width="15.75" customWidth="1"/>
+    <col min="2" max="2" width="16.75" customWidth="1"/>
+    <col min="3" max="3" width="15.75" customWidth="1"/>
+    <col min="4" max="4" width="18.125" customWidth="1"/>
+    <col min="5" max="5" width="20.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="27.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="27.4" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -544,7 +538,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -561,126 +555,126 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -689,9 +683,12 @@
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C4 C6:C1048576" xr:uid="{632E850D-EAD0-4075-AEC5-93E397686794}">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C21:C1048576" xr:uid="{632E850D-EAD0-4075-AEC5-93E397686794}">
       <formula1>"BWI,BSC,VI,FISI"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C20" xr:uid="{1503FFDA-29AC-48F6-9924-EC1B6C203D11}">
+      <formula1>"BWI,BSC,VI,FISI,LLB,PUMA,QE3,QE2,KFB,VFAK"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>